<commit_message>
docs: diversify vessel profiles and voyage profiles
</commit_message>
<xml_diff>
--- a/data/raw/Voyage Estimate.xlsx
+++ b/data/raw/Voyage Estimate.xlsx
@@ -13,10 +13,10 @@
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{35EDC73C-33C3-480C-80C3-EA22C18B9248}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="AQABA" sheetId="2" r:id="rId2"/>
-    <sheet name="Sby" sheetId="3" r:id="rId3"/>
-    <sheet name="Godau" sheetId="4" r:id="rId4"/>
+    <sheet name="Bontang-Mundra" sheetId="1" r:id="rId1"/>
+    <sheet name="Bontang-Davao" sheetId="2" r:id="rId2"/>
+    <sheet name="Bontang-Bangkok" sheetId="3" r:id="rId3"/>
+    <sheet name="Bontang-Hai Phong" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -876,20 +876,20 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B3" s="20" t="s">
-        <v>0</v>
+      <c r="B3" s="20" t="str">
+        <v>HS36</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="1">
-        <v>12</v>
+      <c r="D3" s="1" t="n">
+        <v>11.5</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="1">
-        <v>1956</v>
+      <c r="F3" s="1" t="n">
+        <v>3906</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>5</v>
@@ -903,14 +903,14 @@
       <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="1">
-        <v>14</v>
+      <c r="D4" s="1" t="n">
+        <v>12.5</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="1">
-        <v>1956</v>
+      <c r="F4" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>6</v>
@@ -922,8 +922,9 @@
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B5" s="35" t="s">
-        <v>60</v>
+      <c r="B5" s="35" t="str">
+        <v>UREA GRANULAR BULK
+Asumsi demo</v>
       </c>
       <c r="C5" s="36"/>
       <c r="D5" s="36"/>
@@ -951,15 +952,15 @@
       <c r="G6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="1">
-        <v>25</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0.1</v>
+      <c r="H6" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>0.12</v>
       </c>
       <c r="J6" s="3">
-        <f>0.7*0.1*2000*24/1000</f>
-        <v>3.359999999999999</v>
+        <f>0.7*0.1*1500*24/1000</f>
+        <v>2.5199999999999996</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
@@ -971,11 +972,11 @@
       <c r="G7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="1">
-        <v>23</v>
-      </c>
-      <c r="I7" s="1">
-        <v>0.1</v>
+      <c r="H7" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>0.12</v>
       </c>
       <c r="J7" s="1"/>
     </row>
@@ -1001,41 +1002,44 @@
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B9" s="17" t="s">
-        <v>57</v>
+      <c r="B9" s="17" t="str">
+        <v>BONTANG - MUNDRA</v>
       </c>
       <c r="C9" s="37"/>
       <c r="D9" s="37"/>
       <c r="E9" s="37"/>
       <c r="F9" s="18"/>
       <c r="G9" s="1">
-        <v>1956</v>
+        <f>F3</f>
+        <v>3906</v>
       </c>
       <c r="H9" s="5">
         <f>G9/D3/24</f>
-        <v>6.791666666666667</v>
+        <v>14.152173913043478</v>
       </c>
       <c r="I9" s="6">
         <f>H9*H6</f>
-        <v>169.79166666666669</v>
+        <v>240.58695652173913</v>
       </c>
       <c r="J9" s="6">
         <f>I6*H9</f>
-        <v>0.6791666666666667</v>
+        <v>1.6982608695652173</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B10" s="17" t="s">
-        <v>65</v>
+      <c r="B10" s="17" t="str">
+        <v>RETURN LEG EXCLUDED</v>
       </c>
       <c r="C10" s="37"/>
       <c r="D10" s="37"/>
       <c r="E10" s="37"/>
       <c r="F10" s="18"/>
-      <c r="G10" s="1">
-        <v>1956</v>
-      </c>
-      <c r="H10" s="5"/>
+      <c r="G10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I10" s="6">
         <f>H10*H7</f>
         <v>0</v>
@@ -1046,17 +1050,22 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B11" s="16" t="s">
-        <v>19</v>
+      <c r="B11" s="16" t="str">
+        <v>Waiting (days)</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
       <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
+      <c r="H11" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
+      <c r="J11" s="1">
+        <f>H11*J6</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
@@ -1067,28 +1076,28 @@
       </c>
       <c r="D12" s="5">
         <f>D20/5000</f>
-        <v>6.7721999999999998</v>
+        <v>6</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>59</v>
       </c>
       <c r="F12" s="5">
-        <f>D20/6000</f>
-        <v>5.6435000000000004</v>
+        <f>D20/5000</f>
+        <v>6</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="6">
         <f>D12+F12</f>
-        <v>12.415700000000001</v>
+        <v>12</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
-      <c r="K12">
-        <v>11000</v>
+      <c r="K12" t="n">
+        <v>14500</v>
       </c>
       <c r="L12" s="10">
-        <f>K12*(H9+D12+F12)</f>
-        <v>211281.03333333333</v>
+        <f>K12*H13</f>
+        <v>379206.52173913043</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.35">
@@ -1102,7 +1111,7 @@
       <c r="G13" s="1"/>
       <c r="H13" s="11">
         <f>SUM(H9:H12)</f>
-        <v>19.207366666666669</v>
+        <v>26.152173913043477</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
@@ -1141,8 +1150,8 @@
       <c r="B16" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="20">
-        <v>36009</v>
+      <c r="C16" s="20" t="n">
+        <v>36000</v>
       </c>
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
@@ -1170,8 +1179,8 @@
       <c r="C18" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="20">
-        <v>1648</v>
+      <c r="D18" s="20" t="n">
+        <v>1600</v>
       </c>
       <c r="E18" s="20"/>
       <c r="F18" s="20"/>
@@ -1196,13 +1205,12 @@
       <c r="J19" s="20"/>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B20" s="29" t="s">
-        <v>27</v>
+      <c r="B20" s="29" t="str">
+        <v>Cargo for estimate</v>
       </c>
       <c r="C20" s="30"/>
-      <c r="D20" s="34">
-        <f>C16-D18-D19</f>
-        <v>33861</v>
+      <c r="D20" s="34" t="n">
+        <v>30000</v>
       </c>
       <c r="E20" s="32"/>
       <c r="F20" s="20"/>
@@ -1270,74 +1278,81 @@
       <c r="D24" s="25"/>
       <c r="E24" s="33">
         <f>I9</f>
-        <v>169.79166666666669</v>
+        <v>240.58695652173913</v>
       </c>
       <c r="F24" s="20"/>
-      <c r="G24" s="20">
-        <v>547.5</v>
+      <c r="G24" s="20" t="n">
+        <v>458</v>
       </c>
       <c r="H24" s="20"/>
       <c r="I24" s="7">
         <f>E24*G24</f>
-        <v>92960.937500000015</v>
+        <v>110188.82608695651</v>
       </c>
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B25" s="16"/>
-      <c r="C25" s="29" t="s">
-        <v>62</v>
+      <c r="C25" s="29" t="str">
+        <v>BONTANG</v>
       </c>
       <c r="D25" s="30"/>
       <c r="E25" s="20">
         <v>0</v>
       </c>
       <c r="F25" s="20"/>
-      <c r="G25" s="20">
-        <v>547.5</v>
+      <c r="G25" s="20" t="n">
+        <v>458</v>
       </c>
       <c r="H25" s="20"/>
       <c r="I25" s="7">
-        <f t="shared" ref="I25:I28" si="0">E25*G25</f>
+        <f>E25*G25</f>
         <v>0</v>
       </c>
       <c r="J25" s="1"/>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B26" s="16"/>
-      <c r="C26" s="29" t="s">
-        <v>63</v>
+      <c r="C26" s="29" t="str">
+        <v>MUNDRA</v>
       </c>
       <c r="D26" s="30"/>
       <c r="E26" s="20">
         <v>0</v>
       </c>
       <c r="F26" s="20"/>
-      <c r="G26" s="20">
-        <v>547.5</v>
+      <c r="G26" s="20" t="n">
+        <v>458</v>
       </c>
       <c r="H26" s="20"/>
       <c r="I26" s="7">
-        <f t="shared" si="0"/>
+        <f>E26*G26</f>
         <v>0</v>
       </c>
       <c r="J26" s="4">
         <f>SUM(I24:I26)</f>
-        <v>92960.937500000015</v>
+        <v>110188.82608695651</v>
       </c>
     </row>
     <row r="27" spans="2:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="B27" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="C27" s="2"/>
+      <c r="C27" s="2" t="str">
+        <v>Waiting</v>
+      </c>
       <c r="D27" s="2"/>
-      <c r="E27" s="1"/>
+      <c r="E27" s="1">
+        <f>J11</f>
+        <v>0</v>
+      </c>
       <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
+      <c r="G27" s="1" t="n">
+        <v>902</v>
+      </c>
       <c r="H27" s="1"/>
       <c r="I27" s="7">
-        <f t="shared" si="0"/>
+        <f>E27*G27</f>
         <v>0</v>
       </c>
       <c r="J27" s="1"/>
@@ -1350,62 +1365,62 @@
       <c r="D28" s="25"/>
       <c r="E28" s="26">
         <f>J9</f>
-        <v>0.6791666666666667</v>
+        <v>1.6982608695652173</v>
       </c>
       <c r="F28" s="26"/>
-      <c r="G28" s="20">
-        <v>676</v>
+      <c r="G28" s="20" t="n">
+        <v>902</v>
       </c>
       <c r="H28" s="20"/>
       <c r="I28" s="7">
-        <f t="shared" si="0"/>
-        <v>459.11666666666667</v>
+        <f>E28*G28</f>
+        <v>1531.831304347826</v>
       </c>
       <c r="J28" s="1"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B29" s="25"/>
-      <c r="C29" s="25" t="s">
-        <v>62</v>
+      <c r="C29" s="25" t="str">
+        <v>BONTANG</v>
       </c>
       <c r="D29" s="25"/>
       <c r="E29" s="27">
         <f>J6*D12</f>
-        <v>22.754591999999992</v>
+        <v>15.119999999999997</v>
       </c>
       <c r="F29" s="28"/>
-      <c r="G29" s="34">
-        <v>676</v>
+      <c r="G29" s="34" t="n">
+        <v>902</v>
       </c>
       <c r="H29" s="32"/>
       <c r="I29" s="6">
         <f>E29*G29</f>
-        <v>15382.104191999995</v>
+        <v>13638.239999999998</v>
       </c>
       <c r="J29" s="1"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B30" s="25"/>
-      <c r="C30" s="29" t="s">
-        <v>63</v>
+      <c r="C30" s="29" t="str">
+        <v>MUNDRA</v>
       </c>
       <c r="D30" s="30"/>
       <c r="E30" s="31">
         <f>J6*F12</f>
-        <v>18.962159999999997</v>
+        <v>15.119999999999997</v>
       </c>
       <c r="F30" s="32"/>
-      <c r="G30" s="20">
-        <v>676</v>
+      <c r="G30" s="20" t="n">
+        <v>902</v>
       </c>
       <c r="H30" s="20"/>
       <c r="I30" s="6">
         <f>E30*G30</f>
-        <v>12818.420159999998</v>
+        <v>13638.239999999998</v>
       </c>
       <c r="J30" s="4">
-        <f>SUM(I28:I30)</f>
-        <v>28659.641018666662</v>
+        <f>SUM(I27:I30)</f>
+        <v>28808.311304347822</v>
       </c>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.35">
@@ -1444,8 +1459,13 @@
       <c r="F33" s="16"/>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1"/>
+      <c r="I33" s="1" t="n">
+        <v>80000</v>
+      </c>
+      <c r="J33" s="1">
+        <f>SUM(I33:I37)</f>
+        <v>200000</v>
+      </c>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B34" s="16" t="s">
@@ -1457,7 +1477,9 @@
       <c r="F34" s="16"/>
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
-      <c r="I34" s="1"/>
+      <c r="I34" s="1" t="n">
+        <v>120000</v>
+      </c>
       <c r="J34" s="1"/>
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.35">
@@ -1470,7 +1492,9 @@
       <c r="F35" s="16"/>
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
-      <c r="I35" s="1"/>
+      <c r="I35" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="J35" s="1"/>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.35">
@@ -1483,7 +1507,9 @@
       <c r="F36" s="16"/>
       <c r="G36" s="16"/>
       <c r="H36" s="16"/>
-      <c r="I36" s="1"/>
+      <c r="I36" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="J36" s="1"/>
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.35">
@@ -1496,7 +1522,9 @@
       <c r="F37" s="16"/>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
-      <c r="I37" s="1"/>
+      <c r="I37" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="J37" s="1"/>
     </row>
     <row r="38" spans="2:11" x14ac:dyDescent="0.35">
@@ -1512,11 +1540,11 @@
       <c r="I38" s="20"/>
       <c r="J38" s="8">
         <f>SUM(J24:J37)</f>
-        <v>121620.57851866668</v>
+        <v>338997.13739130436</v>
       </c>
       <c r="K38" s="9">
-        <f>J38/30000</f>
-        <v>4.0540192839555562</v>
+        <f>J38/B41</f>
+        <v>11.299904579710146</v>
       </c>
     </row>
     <row r="39" spans="2:11" x14ac:dyDescent="0.35">
@@ -1555,26 +1583,28 @@
     </row>
     <row r="41" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B41" s="16">
+        <f>D20</f>
         <v>30000</v>
       </c>
       <c r="C41" s="16"/>
       <c r="D41" s="16">
-        <v>15</v>
+        <f>ROUNDUP((J38+K12*H13)/B41,4)</f>
+        <v>23.9402</v>
       </c>
       <c r="E41" s="16"/>
       <c r="F41" s="16">
         <f>B41*D41</f>
-        <v>450000</v>
+        <v>718206</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16">
-        <f>F41*3.75%</f>
-        <v>16875</v>
+        <f>F41*0%</f>
+        <v>0</v>
       </c>
       <c r="I41" s="16"/>
       <c r="J41" s="1">
         <f>F41-H41</f>
-        <v>433125</v>
+        <v>718206</v>
       </c>
     </row>
     <row r="42" spans="2:11" x14ac:dyDescent="0.35">
@@ -1614,29 +1644,29 @@
     <row r="44" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B44" s="19">
         <f>F41-J38</f>
-        <v>328379.42148133332</v>
+        <v>379208.86260869564</v>
       </c>
       <c r="C44" s="20"/>
       <c r="D44" s="21">
         <f>F41/H13</f>
-        <v>23428.510935908267</v>
+        <v>27462.57356608479</v>
       </c>
       <c r="E44" s="21"/>
-      <c r="F44" s="20">
-        <v>5612</v>
+      <c r="F44" s="20" t="n">
+        <v>4800</v>
       </c>
       <c r="G44" s="20"/>
       <c r="H44" s="4">
         <f>J41/H13</f>
-        <v>22549.941775811709</v>
+        <v>27462.57356608479</v>
       </c>
       <c r="I44" s="8">
         <f>J38/H13</f>
-        <v>6331.9756752357171</v>
+        <v>12962.484056525354</v>
       </c>
       <c r="J44" s="8">
         <f>H44-F44-I44</f>
-        <v>10605.966100575992</v>
+        <v>9700.089509559435</v>
       </c>
     </row>
   </sheetData>
@@ -1727,20 +1757,20 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B3" s="20" t="s">
-        <v>0</v>
+      <c r="B3" s="20" t="str">
+        <v>HS38</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="1">
-        <v>14</v>
+      <c r="D3" s="1" t="n">
+        <v>12.5</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="1">
-        <v>5520</v>
+      <c r="F3" s="1" t="n">
+        <v>697</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>5</v>
@@ -1754,14 +1784,14 @@
       <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="1">
-        <v>15</v>
+      <c r="D4" s="1" t="n">
+        <v>13.5</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="1">
-        <v>5520</v>
+      <c r="F4" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>6</v>
@@ -1773,8 +1803,9 @@
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B5" s="35" t="s">
-        <v>68</v>
+      <c r="B5" s="35" t="str">
+        <v>UREA GRANULAR BULK
+Asumsi demo</v>
       </c>
       <c r="C5" s="36"/>
       <c r="D5" s="36"/>
@@ -1802,15 +1833,15 @@
       <c r="G6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="1">
-        <v>29</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0.1</v>
+      <c r="H6" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>0.15</v>
       </c>
       <c r="J6" s="3">
-        <f>0.7*0.1*2000*24/1000</f>
-        <v>3.359999999999999</v>
+        <f>0.7*0.1*1700*24/1000</f>
+        <v>2.8559999999999994</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
@@ -1822,11 +1853,11 @@
       <c r="G7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="1">
-        <v>25</v>
-      </c>
-      <c r="I7" s="1">
-        <v>0.1</v>
+      <c r="H7" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>0.15</v>
       </c>
       <c r="J7" s="1"/>
     </row>
@@ -1852,8 +1883,8 @@
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B9" s="17" t="s">
-        <v>69</v>
+      <c r="B9" s="17" t="str">
+        <v>BONTANG - DAVAO</v>
       </c>
       <c r="C9" s="37"/>
       <c r="D9" s="37"/>
@@ -1861,29 +1892,35 @@
       <c r="F9" s="18"/>
       <c r="G9" s="1">
         <f>F3</f>
-        <v>5520</v>
+        <v>697</v>
       </c>
       <c r="H9" s="5">
         <f>G9/D3/24</f>
-        <v>16.428571428571427</v>
+        <v>2.3233333333333333</v>
       </c>
       <c r="I9" s="6">
         <f>H9*H6</f>
-        <v>476.42857142857139</v>
+        <v>46.46666666666667</v>
       </c>
       <c r="J9" s="6">
         <f>I6*H9</f>
-        <v>1.6428571428571428</v>
+        <v>0.3485</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B10" s="17"/>
+      <c r="B10" s="17" t="str">
+        <v>RETURN LEG EXCLUDED</v>
+      </c>
       <c r="C10" s="37"/>
       <c r="D10" s="37"/>
       <c r="E10" s="37"/>
       <c r="F10" s="18"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="5"/>
+      <c r="G10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I10" s="6">
         <f>H10*H7</f>
         <v>0</v>
@@ -1894,17 +1931,22 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B11" s="16" t="s">
-        <v>19</v>
+      <c r="B11" s="16" t="str">
+        <v>Waiting (days)</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
       <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
+      <c r="H11" s="1" t="n">
+        <v>0.5</v>
+      </c>
       <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
+      <c r="J11" s="1">
+        <f>H11*J6</f>
+        <v>1.4279999999999997</v>
+      </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
@@ -1914,29 +1956,29 @@
         <v>58</v>
       </c>
       <c r="D12" s="5">
-        <f>D20/10000</f>
-        <v>4.5</v>
+        <f>D20/5000</f>
+        <v>5.6</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>87</v>
       </c>
       <c r="F12" s="5">
-        <f>D20/6000</f>
-        <v>7.5</v>
+        <f>D20/4500</f>
+        <v>6.222222222222222</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="6">
         <f>D12+F12</f>
-        <v>12</v>
+        <v>11.822222222222223</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
-      <c r="K12">
-        <v>11000</v>
+      <c r="K12" t="n">
+        <v>14500</v>
       </c>
       <c r="L12" s="10">
-        <f>K12*(H9+D12+F12)</f>
-        <v>312714.28571428568</v>
+        <f>K12*H13</f>
+        <v>212360.55555555556</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.35">
@@ -1950,7 +1992,7 @@
       <c r="G13" s="1"/>
       <c r="H13" s="11">
         <f>SUM(H9:H12)</f>
-        <v>28.428571428571427</v>
+        <v>14.645555555555557</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
@@ -1989,8 +2031,8 @@
       <c r="B16" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="20">
-        <v>58000</v>
+      <c r="C16" s="20" t="n">
+        <v>38000</v>
       </c>
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
@@ -2018,8 +2060,8 @@
       <c r="C18" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="20">
-        <v>1800</v>
+      <c r="D18" s="20" t="n">
+        <v>1700</v>
       </c>
       <c r="E18" s="20"/>
       <c r="F18" s="20"/>
@@ -2044,12 +2086,12 @@
       <c r="J19" s="20"/>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B20" s="29" t="s">
-        <v>27</v>
+      <c r="B20" s="29" t="str">
+        <v>Cargo for estimate</v>
       </c>
       <c r="C20" s="30"/>
-      <c r="D20" s="34">
-        <v>45000</v>
+      <c r="D20" s="34" t="n">
+        <v>28000</v>
       </c>
       <c r="E20" s="32"/>
       <c r="F20" s="20"/>
@@ -2117,75 +2159,82 @@
       <c r="D24" s="25"/>
       <c r="E24" s="33">
         <f>I9</f>
-        <v>476.42857142857139</v>
+        <v>46.46666666666667</v>
       </c>
       <c r="F24" s="20"/>
-      <c r="G24" s="20">
-        <v>568</v>
+      <c r="G24" s="20" t="n">
+        <v>458</v>
       </c>
       <c r="H24" s="20"/>
       <c r="I24" s="7">
         <f>E24*G24</f>
-        <v>270611.42857142852</v>
+        <v>21281.733333333334</v>
       </c>
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B25" s="16"/>
-      <c r="C25" s="29" t="s">
-        <v>62</v>
+      <c r="C25" s="29" t="str">
+        <v>BONTANG</v>
       </c>
       <c r="D25" s="30"/>
       <c r="E25" s="20">
         <v>0</v>
       </c>
       <c r="F25" s="20"/>
-      <c r="G25" s="20">
-        <v>568</v>
+      <c r="G25" s="20" t="n">
+        <v>458</v>
       </c>
       <c r="H25" s="20"/>
       <c r="I25" s="7">
-        <f t="shared" ref="I25:I28" si="0">E25*G25</f>
+        <f>E25*G25</f>
         <v>0</v>
       </c>
       <c r="J25" s="1"/>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B26" s="16"/>
-      <c r="C26" s="29" t="s">
-        <v>63</v>
+      <c r="C26" s="29" t="str">
+        <v>DAVAO</v>
       </c>
       <c r="D26" s="30"/>
       <c r="E26" s="20">
         <v>0</v>
       </c>
       <c r="F26" s="20"/>
-      <c r="G26" s="20">
-        <v>568</v>
+      <c r="G26" s="20" t="n">
+        <v>458</v>
       </c>
       <c r="H26" s="20"/>
       <c r="I26" s="7">
-        <f t="shared" si="0"/>
+        <f>E26*G26</f>
         <v>0</v>
       </c>
       <c r="J26" s="4">
         <f>SUM(I24:I26)</f>
-        <v>270611.42857142852</v>
+        <v>21281.733333333334</v>
       </c>
     </row>
     <row r="27" spans="2:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="B27" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="C27" s="2"/>
+      <c r="C27" s="2" t="str">
+        <v>Waiting</v>
+      </c>
       <c r="D27" s="2"/>
-      <c r="E27" s="1"/>
+      <c r="E27" s="1">
+        <f>J11</f>
+        <v>1.4279999999999997</v>
+      </c>
       <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
+      <c r="G27" s="1" t="n">
+        <v>902</v>
+      </c>
       <c r="H27" s="1"/>
       <c r="I27" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>E27*G27</f>
+        <v>1288.0559999999998</v>
       </c>
       <c r="J27" s="1"/>
     </row>
@@ -2197,62 +2246,62 @@
       <c r="D28" s="25"/>
       <c r="E28" s="26">
         <f>J9</f>
-        <v>1.6428571428571428</v>
+        <v>0.3485</v>
       </c>
       <c r="F28" s="26"/>
-      <c r="G28" s="20">
-        <v>701</v>
+      <c r="G28" s="20" t="n">
+        <v>902</v>
       </c>
       <c r="H28" s="20"/>
       <c r="I28" s="7">
-        <f t="shared" si="0"/>
-        <v>1151.6428571428571</v>
+        <f>E28*G28</f>
+        <v>314.347</v>
       </c>
       <c r="J28" s="1"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B29" s="25"/>
-      <c r="C29" s="25" t="s">
-        <v>62</v>
+      <c r="C29" s="25" t="str">
+        <v>BONTANG</v>
       </c>
       <c r="D29" s="25"/>
       <c r="E29" s="27">
         <f>J6*D12</f>
-        <v>15.119999999999996</v>
+        <v>15.993599999999995</v>
       </c>
       <c r="F29" s="28"/>
-      <c r="G29" s="20">
-        <v>701</v>
+      <c r="G29" s="20" t="n">
+        <v>902</v>
       </c>
       <c r="H29" s="20"/>
       <c r="I29" s="6">
         <f>E29*G29</f>
-        <v>10599.119999999997</v>
+        <v>14426.227199999996</v>
       </c>
       <c r="J29" s="1"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B30" s="25"/>
-      <c r="C30" s="29" t="s">
-        <v>63</v>
+      <c r="C30" s="29" t="str">
+        <v>DAVAO</v>
       </c>
       <c r="D30" s="30"/>
       <c r="E30" s="31">
         <f>J6*F12</f>
-        <v>25.199999999999992</v>
+        <v>17.770666666666664</v>
       </c>
       <c r="F30" s="32"/>
-      <c r="G30" s="20">
-        <v>701</v>
+      <c r="G30" s="20" t="n">
+        <v>902</v>
       </c>
       <c r="H30" s="20"/>
       <c r="I30" s="6">
         <f>E30*G30</f>
-        <v>17665.199999999993</v>
+        <v>16029.141333333331</v>
       </c>
       <c r="J30" s="4">
-        <f>SUM(I28:I30)</f>
-        <v>29415.962857142847</v>
+        <f>SUM(I27:I30)</f>
+        <v>32057.771533333325</v>
       </c>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.35">
@@ -2291,9 +2340,12 @@
       <c r="F33" s="16"/>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
-      <c r="I33" s="1"/>
+      <c r="I33" s="1" t="n">
+        <v>45000</v>
+      </c>
       <c r="J33" s="22">
-        <v>200000</v>
+        <f>SUM(I33:I37)</f>
+        <v>90000</v>
       </c>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.35">
@@ -2306,7 +2358,9 @@
       <c r="F34" s="16"/>
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
-      <c r="I34" s="1"/>
+      <c r="I34" s="1" t="n">
+        <v>40000</v>
+      </c>
       <c r="J34" s="23"/>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.35">
@@ -2319,7 +2373,9 @@
       <c r="F35" s="16"/>
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
-      <c r="I35" s="1"/>
+      <c r="I35" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="J35" s="23"/>
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.35">
@@ -2332,7 +2388,9 @@
       <c r="F36" s="16"/>
       <c r="G36" s="16"/>
       <c r="H36" s="16"/>
-      <c r="I36" s="1"/>
+      <c r="I36" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="J36" s="23"/>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.35">
@@ -2345,7 +2403,9 @@
       <c r="F37" s="16"/>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
-      <c r="I37" s="1"/>
+      <c r="I37" s="1" t="n">
+        <v>5000</v>
+      </c>
       <c r="J37" s="24"/>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.35">
@@ -2361,13 +2421,14 @@
       <c r="I38" s="20"/>
       <c r="J38" s="8">
         <f>SUM(J24:J37)</f>
-        <v>500027.39142857137</v>
-      </c>
-      <c r="K38" t="s">
-        <v>82</v>
+        <v>143339.50486666666</v>
+      </c>
+      <c r="K38" t="str">
+        <v>Target/day</v>
       </c>
       <c r="L38">
-        <v>13000</v>
+        <f>K12</f>
+        <v>14500</v>
       </c>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.35">
@@ -2382,12 +2443,12 @@
       <c r="H39" s="16"/>
       <c r="I39" s="16"/>
       <c r="J39" s="16"/>
-      <c r="K39" t="s">
-        <v>76</v>
+      <c r="K39" t="str">
+        <v>Voyage cost/MT</v>
       </c>
       <c r="L39" s="9">
-        <f>J38/46000</f>
-        <v>10.870160683229813</v>
+        <f>J38/B41</f>
+        <v>5.11926803095238</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.35">
@@ -2410,43 +2471,45 @@
       <c r="J40" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K40" t="s">
-        <v>77</v>
+      <c r="K40" t="str">
+        <v>Target/day part</v>
       </c>
       <c r="L40" s="10">
-        <f>L38*(H13)/45000</f>
-        <v>8.2126984126984137</v>
+        <f>L38*H13/B41</f>
+        <v>7.584305555555556</v>
       </c>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B41" s="16">
-        <v>45000</v>
+        <f>D20</f>
+        <v>28000</v>
       </c>
       <c r="C41" s="16"/>
       <c r="D41" s="16">
-        <v>20</v>
+        <f>ROUNDUP((J38+K12*H13)/B41,4)</f>
+        <v>12.7036</v>
       </c>
       <c r="E41" s="16"/>
       <c r="F41" s="16">
         <f>B41*D41</f>
-        <v>900000</v>
+        <v>355700.8</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16">
-        <f>F41*2.5%</f>
-        <v>22500</v>
+        <f>F41*0%</f>
+        <v>0</v>
       </c>
       <c r="I41" s="16"/>
       <c r="J41" s="1">
         <f>F41-H41</f>
-        <v>877500</v>
+        <v>355700.8</v>
       </c>
       <c r="K41" t="s">
         <v>75</v>
       </c>
       <c r="L41" s="12">
         <f>SUM(L39:L40)</f>
-        <v>19.082859095928228</v>
+        <v>12.703573586507936</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.35">
@@ -2463,7 +2526,8 @@
         <v>80</v>
       </c>
       <c r="L42">
-        <v>20</v>
+        <f>D41</f>
+        <v>12.7036</v>
       </c>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.35">
@@ -2488,64 +2552,64 @@
       <c r="J43" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="K43" t="s">
-        <v>78</v>
+      <c r="K43" t="str">
+        <v>Net / MT</v>
       </c>
       <c r="L43" s="10">
-        <f>L42-L41</f>
-        <v>0.91714090407177196</v>
+        <f>J44*H13/B41</f>
+        <v>4.86444308015873</v>
       </c>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B44" s="19">
         <f>F41-J38</f>
-        <v>399972.60857142863</v>
+        <v>212361.29513333333</v>
       </c>
       <c r="C44" s="20"/>
       <c r="D44" s="21">
         <f>F41/H13</f>
-        <v>31658.291457286436</v>
+        <v>24287.286245353156</v>
       </c>
       <c r="E44" s="21"/>
-      <c r="F44" s="20">
-        <v>5612</v>
+      <c r="F44" s="20" t="n">
+        <v>5200</v>
       </c>
       <c r="G44" s="20"/>
       <c r="H44" s="4">
         <f>J41/H13</f>
-        <v>30866.834170854272</v>
+        <v>24287.286245353156</v>
       </c>
       <c r="I44" s="8">
         <f>J38/H13</f>
-        <v>17588.903216080402</v>
+        <v>9787.235746908427</v>
       </c>
       <c r="J44" s="8">
         <f>H44-F44-I44</f>
-        <v>7665.9309547738703</v>
-      </c>
-      <c r="K44" t="s">
-        <v>79</v>
+        <v>9300.050498444729</v>
+      </c>
+      <c r="K44" t="str">
+        <v>Total net</v>
       </c>
       <c r="L44" s="10">
-        <f>L43*45000</f>
-        <v>41271.340683229741</v>
+        <f>L43*B41</f>
+        <v>136204.40624444443</v>
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="K45" t="s">
-        <v>81</v>
+      <c r="K45" t="str">
+        <v>Total net IDR</v>
       </c>
       <c r="L45" s="10">
         <f>L44*15800</f>
-        <v>652087182.79502988</v>
+        <v>2152029618.662222</v>
       </c>
       <c r="M45" s="10">
-        <f>L38*15*15800</f>
-        <v>3081000000</v>
+        <f>F44*H13*15800</f>
+        <v>1203278844.4444444</v>
       </c>
       <c r="N45" s="15">
         <f>L45/M45</f>
-        <v>0.2116479009396397</v>
+        <v>1.7884712497009096</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.35">
@@ -2553,8 +2617,8 @@
         <v>83</v>
       </c>
       <c r="L46">
-        <f>L42*1.25%*B41</f>
-        <v>11250</v>
+        <f>L42*0%*B41</f>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.35">
@@ -2563,7 +2627,7 @@
       </c>
       <c r="L47" s="13">
         <f>L46*15800</f>
-        <v>177750000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.35">
@@ -2571,8 +2635,8 @@
         <v>85</v>
       </c>
       <c r="L48">
-        <f>L42*2.5%*B41</f>
-        <v>22500</v>
+        <f>L42*0%*B41</f>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="11:12" x14ac:dyDescent="0.35">
@@ -2581,7 +2645,7 @@
       </c>
       <c r="L49" s="13">
         <f>L48*15800</f>
-        <v>355500000</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2671,20 +2735,20 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B3" s="20" t="s">
-        <v>0</v>
+      <c r="B3" s="20" t="str">
+        <v>SUP54</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="1" t="n">
         <v>12</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="1">
-        <v>237</v>
+      <c r="F3" s="1" t="n">
+        <v>1751</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>5</v>
@@ -2698,13 +2762,15 @@
       <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="1">
-        <v>14</v>
+      <c r="D4" s="1" t="n">
+        <v>13</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="1"/>
+      <c r="F4" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G4" s="1" t="s">
         <v>6</v>
       </c>
@@ -2715,8 +2781,9 @@
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B5" s="35" t="s">
-        <v>68</v>
+      <c r="B5" s="35" t="str">
+        <v>UREA GRANULAR BULK
+Asumsi demo</v>
       </c>
       <c r="C5" s="36"/>
       <c r="D5" s="36"/>
@@ -2744,11 +2811,11 @@
       <c r="G6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="1">
-        <v>25</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0.1</v>
+      <c r="H6" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>0.18</v>
       </c>
       <c r="J6" s="3">
         <f>0.7*0.1*2000*24/1000</f>
@@ -2764,11 +2831,11 @@
       <c r="G7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="1">
-        <v>21</v>
-      </c>
-      <c r="I7" s="1">
-        <v>0.1</v>
+      <c r="H7" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>0.18</v>
       </c>
       <c r="J7" s="1"/>
     </row>
@@ -2794,8 +2861,8 @@
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B9" s="17" t="s">
-        <v>69</v>
+      <c r="B9" s="17" t="str">
+        <v>BONTANG - BANGKOK</v>
       </c>
       <c r="C9" s="37"/>
       <c r="D9" s="37"/>
@@ -2803,29 +2870,35 @@
       <c r="F9" s="18"/>
       <c r="G9" s="1">
         <f>F3</f>
-        <v>237</v>
+        <v>1751</v>
       </c>
       <c r="H9" s="5">
         <f>G9/D3/24</f>
-        <v>0.82291666666666663</v>
+        <v>6.079861111111111</v>
       </c>
       <c r="I9" s="6">
         <f>H9*H6</f>
-        <v>20.572916666666664</v>
+        <v>145.91666666666666</v>
       </c>
       <c r="J9" s="6">
         <f>I6*H9</f>
-        <v>8.2291666666666666E-2</v>
+        <v>1.0943749999999999</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B10" s="17"/>
+      <c r="B10" s="17" t="str">
+        <v>RETURN LEG EXCLUDED</v>
+      </c>
       <c r="C10" s="37"/>
       <c r="D10" s="37"/>
       <c r="E10" s="37"/>
       <c r="F10" s="18"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="5"/>
+      <c r="G10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I10" s="6">
         <f>H10*H7</f>
         <v>0</v>
@@ -2836,17 +2909,22 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B11" s="16" t="s">
-        <v>19</v>
+      <c r="B11" s="16" t="str">
+        <v>Waiting (days)</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
       <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
+      <c r="H11" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
+      <c r="J11" s="1">
+        <f>H11*J6</f>
+        <v>3.359999999999999</v>
+      </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
@@ -2857,28 +2935,28 @@
       </c>
       <c r="D12" s="5">
         <f>D20/5000</f>
-        <v>5</v>
+        <v>6.4</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>59</v>
       </c>
       <c r="F12" s="5">
-        <f>D20/5000</f>
-        <v>5</v>
+        <f>D20/4000</f>
+        <v>8</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="6">
         <f>D12+F12</f>
-        <v>10</v>
+        <v>14.4</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
-      <c r="K12">
-        <v>11000</v>
+      <c r="K12" t="n">
+        <v>17500</v>
       </c>
       <c r="L12" s="10">
-        <f>K12*(H9+D12+F12)</f>
-        <v>119052.08333333334</v>
+        <f>K12*H13</f>
+        <v>375897.5694444445</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.35">
@@ -2892,7 +2970,7 @@
       <c r="G13" s="1"/>
       <c r="H13" s="11">
         <f>SUM(H9:H12)</f>
-        <v>10.822916666666666</v>
+        <v>21.479861111111113</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
@@ -2931,8 +3009,8 @@
       <c r="B16" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="20">
-        <v>58000</v>
+      <c r="C16" s="20" t="n">
+        <v>54000</v>
       </c>
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
@@ -2960,7 +3038,7 @@
       <c r="C18" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="20" t="n">
         <v>1800</v>
       </c>
       <c r="E18" s="20"/>
@@ -2986,12 +3064,12 @@
       <c r="J19" s="20"/>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B20" s="29" t="s">
-        <v>27</v>
+      <c r="B20" s="29" t="str">
+        <v>Cargo for estimate</v>
       </c>
       <c r="C20" s="30"/>
-      <c r="D20" s="34">
-        <v>25000</v>
+      <c r="D20" s="34" t="n">
+        <v>32000</v>
       </c>
       <c r="E20" s="32"/>
       <c r="F20" s="20"/>
@@ -3059,71 +3137,82 @@
       <c r="D24" s="25"/>
       <c r="E24" s="33">
         <f>I9</f>
-        <v>20.572916666666664</v>
+        <v>145.91666666666666</v>
       </c>
       <c r="F24" s="20"/>
-      <c r="G24" s="20">
-        <v>547.5</v>
+      <c r="G24" s="20" t="n">
+        <v>458</v>
       </c>
       <c r="H24" s="20"/>
       <c r="I24" s="7">
         <f>E24*G24</f>
-        <v>11263.671874999998</v>
+        <v>66829.83333333333</v>
       </c>
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B25" s="16"/>
-      <c r="C25" s="29"/>
+      <c r="C25" s="29" t="str">
+        <v>BONTANG</v>
+      </c>
       <c r="D25" s="30"/>
       <c r="E25" s="20">
         <v>0</v>
       </c>
       <c r="F25" s="20"/>
-      <c r="G25" s="20">
-        <v>547.5</v>
+      <c r="G25" s="20" t="n">
+        <v>458</v>
       </c>
       <c r="H25" s="20"/>
       <c r="I25" s="7">
-        <f t="shared" ref="I25:I28" si="0">E25*G25</f>
+        <f>E25*G25</f>
         <v>0</v>
       </c>
       <c r="J25" s="1"/>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B26" s="16"/>
-      <c r="C26" s="29"/>
+      <c r="C26" s="29" t="str">
+        <v>BANGKOK</v>
+      </c>
       <c r="D26" s="30"/>
       <c r="E26" s="20">
         <v>0</v>
       </c>
       <c r="F26" s="20"/>
-      <c r="G26" s="20">
-        <v>547.5</v>
+      <c r="G26" s="20" t="n">
+        <v>458</v>
       </c>
       <c r="H26" s="20"/>
       <c r="I26" s="7">
-        <f t="shared" si="0"/>
+        <f>E26*G26</f>
         <v>0</v>
       </c>
       <c r="J26" s="4">
         <f>SUM(I24:I26)</f>
-        <v>11263.671874999998</v>
+        <v>66829.83333333333</v>
       </c>
     </row>
     <row r="27" spans="2:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="B27" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="C27" s="2"/>
+      <c r="C27" s="2" t="str">
+        <v>Waiting</v>
+      </c>
       <c r="D27" s="2"/>
-      <c r="E27" s="1"/>
+      <c r="E27" s="1">
+        <f>J11</f>
+        <v>3.359999999999999</v>
+      </c>
       <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
+      <c r="G27" s="1" t="n">
+        <v>902</v>
+      </c>
       <c r="H27" s="1"/>
       <c r="I27" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>E27*G27</f>
+        <v>3030.719999999999</v>
       </c>
       <c r="J27" s="1"/>
     </row>
@@ -3135,62 +3224,62 @@
       <c r="D28" s="25"/>
       <c r="E28" s="26">
         <f>J9</f>
-        <v>8.2291666666666666E-2</v>
+        <v>1.0943749999999999</v>
       </c>
       <c r="F28" s="26"/>
-      <c r="G28" s="20">
-        <v>676</v>
+      <c r="G28" s="20" t="n">
+        <v>902</v>
       </c>
       <c r="H28" s="20"/>
       <c r="I28" s="7">
-        <f t="shared" si="0"/>
-        <v>55.629166666666663</v>
+        <f>E28*G28</f>
+        <v>987.1262499999999</v>
       </c>
       <c r="J28" s="1"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B29" s="25"/>
-      <c r="C29" s="25" t="s">
-        <v>62</v>
+      <c r="C29" s="25" t="str">
+        <v>BONTANG</v>
       </c>
       <c r="D29" s="25"/>
       <c r="E29" s="27">
         <f>J6*D12</f>
-        <v>16.799999999999994</v>
+        <v>21.503999999999994</v>
       </c>
       <c r="F29" s="28"/>
-      <c r="G29" s="34">
-        <v>676</v>
+      <c r="G29" s="34" t="n">
+        <v>902</v>
       </c>
       <c r="H29" s="32"/>
       <c r="I29" s="6">
         <f>E29*G29</f>
-        <v>11356.799999999996</v>
+        <v>19396.607999999997</v>
       </c>
       <c r="J29" s="1"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B30" s="25"/>
-      <c r="C30" s="29" t="s">
-        <v>63</v>
+      <c r="C30" s="29" t="str">
+        <v>BANGKOK</v>
       </c>
       <c r="D30" s="30"/>
       <c r="E30" s="31">
         <f>J6*F12</f>
-        <v>16.799999999999994</v>
+        <v>26.879999999999992</v>
       </c>
       <c r="F30" s="32"/>
-      <c r="G30" s="20">
-        <v>676</v>
+      <c r="G30" s="20" t="n">
+        <v>902</v>
       </c>
       <c r="H30" s="20"/>
       <c r="I30" s="6">
         <f>E30*G30</f>
-        <v>11356.799999999996</v>
+        <v>24245.75999999999</v>
       </c>
       <c r="J30" s="4">
-        <f>SUM(I28:I30)</f>
-        <v>22769.229166666657</v>
+        <f>SUM(I27:I30)</f>
+        <v>47660.21424999999</v>
       </c>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.35">
@@ -3229,8 +3318,13 @@
       <c r="F33" s="16"/>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1"/>
+      <c r="I33" s="1" t="n">
+        <v>50000</v>
+      </c>
+      <c r="J33" s="1">
+        <f>SUM(I33:I37)</f>
+        <v>120000</v>
+      </c>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="16" t="s">
@@ -3242,7 +3336,9 @@
       <c r="F34" s="16"/>
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
-      <c r="I34" s="1"/>
+      <c r="I34" s="1" t="n">
+        <v>65000</v>
+      </c>
       <c r="J34" s="1"/>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.35">
@@ -3255,7 +3351,9 @@
       <c r="F35" s="16"/>
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
-      <c r="I35" s="1"/>
+      <c r="I35" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="J35" s="1"/>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.35">
@@ -3268,10 +3366,10 @@
       <c r="F36" s="16"/>
       <c r="G36" s="16"/>
       <c r="H36" s="16"/>
-      <c r="I36" s="1"/>
-      <c r="J36" s="1">
-        <v>250000</v>
-      </c>
+      <c r="I36" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="1"/>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="16" t="s">
@@ -3283,7 +3381,9 @@
       <c r="F37" s="16"/>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
-      <c r="I37" s="1"/>
+      <c r="I37" s="1" t="n">
+        <v>5000</v>
+      </c>
       <c r="J37" s="1"/>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.35">
@@ -3299,11 +3399,11 @@
       <c r="I38" s="20"/>
       <c r="J38" s="8">
         <f>SUM(J24:J37)</f>
-        <v>284032.90104166663</v>
+        <v>234490.04758333333</v>
       </c>
       <c r="K38" s="9">
-        <f>J38/46000</f>
-        <v>6.1746282835144921</v>
+        <f>J38/B41</f>
+        <v>7.327813986979167</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.35">
@@ -3319,8 +3419,8 @@
       <c r="I39" s="16"/>
       <c r="J39" s="16"/>
       <c r="K39" s="10">
-        <f>11500*(H13)/25000</f>
-        <v>4.9785416666666666</v>
+        <f>K12*H13/B41</f>
+        <v>11.746799045138891</v>
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.35">
@@ -3345,35 +3445,37 @@
       </c>
       <c r="K40" s="12">
         <f>SUM(K38:K39)</f>
-        <v>11.153169950181159</v>
+        <v>19.07461303211806</v>
       </c>
       <c r="L40" s="13">
         <f>K40*15800</f>
-        <v>176220.08521286232</v>
+        <v>301378.8859074653</v>
       </c>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B41" s="16">
-        <v>46000</v>
+        <f>D20</f>
+        <v>32000</v>
       </c>
       <c r="C41" s="16"/>
       <c r="D41" s="16">
-        <v>20</v>
+        <f>ROUNDUP((J38+K12*H13)/B41,4)</f>
+        <v>19.0747</v>
       </c>
       <c r="E41" s="16"/>
       <c r="F41" s="16">
         <f>B41*D41</f>
-        <v>920000</v>
+        <v>610390.4</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16">
-        <f>F41*3.75%</f>
-        <v>34500</v>
+        <f>F41*0%</f>
+        <v>0</v>
       </c>
       <c r="I41" s="16"/>
       <c r="J41" s="1">
         <f>F41-H41</f>
-        <v>885500</v>
+        <v>610390.4</v>
       </c>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.35">
@@ -3413,29 +3515,29 @@
     <row r="44" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B44" s="19">
         <f>F41-J38</f>
-        <v>635967.09895833337</v>
+        <v>375900.3524166667</v>
       </c>
       <c r="C44" s="20"/>
       <c r="D44" s="21">
         <f>F41/H13</f>
-        <v>85004.812319538018</v>
+        <v>28416.869031069153</v>
       </c>
       <c r="E44" s="21"/>
-      <c r="F44" s="20">
-        <v>5612</v>
+      <c r="F44" s="20" t="n">
+        <v>6100</v>
       </c>
       <c r="G44" s="20"/>
       <c r="H44" s="4">
         <f>J41/H13</f>
-        <v>81817.131857555345</v>
+        <v>28416.869031069153</v>
       </c>
       <c r="I44" s="8">
         <f>J38/H13</f>
-        <v>26243.655919153029</v>
+        <v>10916.73946914099</v>
       </c>
       <c r="J44" s="8">
         <f>H44-F44-I44</f>
-        <v>49961.47593840232</v>
+        <v>11400.129561928163</v>
       </c>
     </row>
   </sheetData>
@@ -3525,20 +3627,20 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B3" s="20" t="s">
-        <v>0</v>
+      <c r="B3" s="20" t="str">
+        <v>SUP58</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="1">
-        <v>12</v>
+      <c r="D3" s="1" t="n">
+        <v>13</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="1">
-        <v>1016</v>
+      <c r="F3" s="1" t="n">
+        <v>1577</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>5</v>
@@ -3552,13 +3654,15 @@
       <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="1" t="n">
         <v>14</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="1"/>
+      <c r="F4" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G4" s="1" t="s">
         <v>6</v>
       </c>
@@ -3569,8 +3673,9 @@
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B5" s="35" t="s">
-        <v>68</v>
+      <c r="B5" s="35" t="str">
+        <v>UREA GRANULAR BULK
+Asumsi demo</v>
       </c>
       <c r="C5" s="36"/>
       <c r="D5" s="36"/>
@@ -3598,15 +3703,15 @@
       <c r="G6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="1">
-        <v>25</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0.1</v>
+      <c r="H6" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>0.2</v>
       </c>
       <c r="J6" s="3">
-        <f>0.7*0.1*2000*24/1000</f>
-        <v>3.359999999999999</v>
+        <f>0.7*0.1*2300*24/1000</f>
+        <v>3.863999999999999</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
@@ -3618,11 +3723,11 @@
       <c r="G7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="1">
-        <v>21</v>
-      </c>
-      <c r="I7" s="1">
-        <v>0.1</v>
+      <c r="H7" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>0.2</v>
       </c>
       <c r="J7" s="1"/>
     </row>
@@ -3648,8 +3753,8 @@
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B9" s="17" t="s">
-        <v>70</v>
+      <c r="B9" s="17" t="str">
+        <v>BONTANG - HAI PHONG</v>
       </c>
       <c r="C9" s="37"/>
       <c r="D9" s="37"/>
@@ -3657,29 +3762,35 @@
       <c r="F9" s="18"/>
       <c r="G9" s="1">
         <f>F3</f>
-        <v>1016</v>
+        <v>1577</v>
       </c>
       <c r="H9" s="5">
         <f>G9/D3/24</f>
-        <v>3.5277777777777781</v>
+        <v>5.05448717948718</v>
       </c>
       <c r="I9" s="6">
         <f>H9*H6</f>
-        <v>88.194444444444457</v>
+        <v>141.52564102564102</v>
       </c>
       <c r="J9" s="6">
         <f>I6*H9</f>
-        <v>0.35277777777777786</v>
+        <v>1.010897435897436</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B10" s="17"/>
+      <c r="B10" s="17" t="str">
+        <v>RETURN LEG EXCLUDED</v>
+      </c>
       <c r="C10" s="37"/>
       <c r="D10" s="37"/>
       <c r="E10" s="37"/>
       <c r="F10" s="18"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="5"/>
+      <c r="G10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I10" s="6">
         <f>H10*H7</f>
         <v>0</v>
@@ -3690,17 +3801,22 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B11" s="16" t="s">
-        <v>19</v>
+      <c r="B11" s="16" t="str">
+        <v>Waiting (days)</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
       <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
+      <c r="H11" s="1" t="n">
+        <v>0.5</v>
+      </c>
       <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
+      <c r="J11" s="1">
+        <f>H11*J6</f>
+        <v>1.9319999999999995</v>
+      </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
@@ -3711,28 +3827,28 @@
       </c>
       <c r="D12" s="5">
         <f>D20/5000</f>
-        <v>5</v>
+        <v>5.8</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>59</v>
       </c>
       <c r="F12" s="5">
         <f>D20/5000</f>
-        <v>5</v>
+        <v>5.8</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="6">
         <f>D12+F12</f>
-        <v>10</v>
+        <v>11.6</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
-      <c r="K12">
-        <v>11000</v>
+      <c r="K12" t="n">
+        <v>17500</v>
       </c>
       <c r="L12" s="10">
-        <f>K12*(H9+D12+F12)</f>
-        <v>148805.55555555556</v>
+        <f>K12*H13</f>
+        <v>300203.5256410256</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.35">
@@ -3746,7 +3862,7 @@
       <c r="G13" s="1"/>
       <c r="H13" s="11">
         <f>SUM(H9:H12)</f>
-        <v>13.527777777777779</v>
+        <v>17.15448717948718</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
@@ -3785,8 +3901,8 @@
       <c r="B16" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="20">
-        <v>47175</v>
+      <c r="C16" s="20" t="n">
+        <v>58000</v>
       </c>
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
@@ -3814,8 +3930,8 @@
       <c r="C18" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="20">
-        <v>1800</v>
+      <c r="D18" s="20" t="n">
+        <v>2000</v>
       </c>
       <c r="E18" s="20"/>
       <c r="F18" s="20"/>
@@ -3840,12 +3956,12 @@
       <c r="J19" s="20"/>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B20" s="29" t="s">
-        <v>27</v>
+      <c r="B20" s="29" t="str">
+        <v>Cargo for estimate</v>
       </c>
       <c r="C20" s="30"/>
-      <c r="D20" s="34">
-        <v>25000</v>
+      <c r="D20" s="34" t="n">
+        <v>29000</v>
       </c>
       <c r="E20" s="32"/>
       <c r="F20" s="20"/>
@@ -3913,71 +4029,82 @@
       <c r="D24" s="25"/>
       <c r="E24" s="33">
         <f>I9</f>
-        <v>88.194444444444457</v>
+        <v>141.52564102564102</v>
       </c>
       <c r="F24" s="20"/>
-      <c r="G24" s="20">
-        <v>547.5</v>
+      <c r="G24" s="20" t="n">
+        <v>458</v>
       </c>
       <c r="H24" s="20"/>
       <c r="I24" s="7">
         <f>E24*G24</f>
-        <v>48286.458333333343</v>
+        <v>64818.743589743586</v>
       </c>
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B25" s="16"/>
-      <c r="C25" s="29"/>
+      <c r="C25" s="29" t="str">
+        <v>BONTANG</v>
+      </c>
       <c r="D25" s="30"/>
       <c r="E25" s="20">
         <v>0</v>
       </c>
       <c r="F25" s="20"/>
-      <c r="G25" s="20">
-        <v>547.5</v>
+      <c r="G25" s="20" t="n">
+        <v>458</v>
       </c>
       <c r="H25" s="20"/>
       <c r="I25" s="7">
-        <f t="shared" ref="I25:I28" si="0">E25*G25</f>
+        <f>E25*G25</f>
         <v>0</v>
       </c>
       <c r="J25" s="1"/>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B26" s="16"/>
-      <c r="C26" s="29"/>
+      <c r="C26" s="29" t="str">
+        <v>HAI PHONG</v>
+      </c>
       <c r="D26" s="30"/>
       <c r="E26" s="20">
         <v>0</v>
       </c>
       <c r="F26" s="20"/>
-      <c r="G26" s="20">
-        <v>547.5</v>
+      <c r="G26" s="20" t="n">
+        <v>458</v>
       </c>
       <c r="H26" s="20"/>
       <c r="I26" s="7">
-        <f t="shared" si="0"/>
+        <f>E26*G26</f>
         <v>0</v>
       </c>
       <c r="J26" s="4">
         <f>SUM(I24:I26)</f>
-        <v>48286.458333333343</v>
+        <v>64818.743589743586</v>
       </c>
     </row>
     <row r="27" spans="2:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="B27" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="C27" s="2"/>
+      <c r="C27" s="2" t="str">
+        <v>Waiting</v>
+      </c>
       <c r="D27" s="2"/>
-      <c r="E27" s="1"/>
+      <c r="E27" s="1">
+        <f>J11</f>
+        <v>1.9319999999999995</v>
+      </c>
       <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
+      <c r="G27" s="1" t="n">
+        <v>902</v>
+      </c>
       <c r="H27" s="1"/>
       <c r="I27" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>E27*G27</f>
+        <v>1742.6639999999995</v>
       </c>
       <c r="J27" s="1"/>
     </row>
@@ -3989,62 +4116,62 @@
       <c r="D28" s="25"/>
       <c r="E28" s="26">
         <f>J9</f>
-        <v>0.35277777777777786</v>
+        <v>1.010897435897436</v>
       </c>
       <c r="F28" s="26"/>
-      <c r="G28" s="20">
-        <v>676</v>
+      <c r="G28" s="20" t="n">
+        <v>902</v>
       </c>
       <c r="H28" s="20"/>
       <c r="I28" s="7">
-        <f t="shared" si="0"/>
-        <v>238.47777777777782</v>
+        <f>E28*G28</f>
+        <v>911.8294871794874</v>
       </c>
       <c r="J28" s="1"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B29" s="25"/>
-      <c r="C29" s="25" t="s">
-        <v>71</v>
+      <c r="C29" s="25" t="str">
+        <v>BONTANG</v>
       </c>
       <c r="D29" s="25"/>
       <c r="E29" s="27">
         <f>J6*D12</f>
-        <v>16.799999999999994</v>
+        <v>22.411199999999994</v>
       </c>
       <c r="F29" s="28"/>
-      <c r="G29" s="34">
-        <v>676</v>
+      <c r="G29" s="34" t="n">
+        <v>902</v>
       </c>
       <c r="H29" s="32"/>
       <c r="I29" s="6">
         <f>E29*G29</f>
-        <v>11356.799999999996</v>
+        <v>20214.902399999995</v>
       </c>
       <c r="J29" s="1"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B30" s="25"/>
-      <c r="C30" s="29" t="s">
-        <v>72</v>
+      <c r="C30" s="29" t="str">
+        <v>HAI PHONG</v>
       </c>
       <c r="D30" s="30"/>
       <c r="E30" s="31">
         <f>J6*F12</f>
-        <v>16.799999999999994</v>
+        <v>22.411199999999994</v>
       </c>
       <c r="F30" s="32"/>
-      <c r="G30" s="20">
-        <v>676</v>
+      <c r="G30" s="20" t="n">
+        <v>902</v>
       </c>
       <c r="H30" s="20"/>
       <c r="I30" s="6">
         <f>E30*G30</f>
-        <v>11356.799999999996</v>
+        <v>20214.902399999995</v>
       </c>
       <c r="J30" s="4">
-        <f>SUM(I28:I30)</f>
-        <v>22952.077777777769</v>
+        <f>SUM(I27:I30)</f>
+        <v>43084.29828717948</v>
       </c>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.35">
@@ -4083,8 +4210,13 @@
       <c r="F33" s="16"/>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1"/>
+      <c r="I33" s="1" t="n">
+        <v>50000</v>
+      </c>
+      <c r="J33" s="1">
+        <f>SUM(I33:I37)</f>
+        <v>110000</v>
+      </c>
     </row>
     <row r="34" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B34" s="16" t="s">
@@ -4096,7 +4228,9 @@
       <c r="F34" s="16"/>
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
-      <c r="I34" s="1"/>
+      <c r="I34" s="1" t="n">
+        <v>55000</v>
+      </c>
       <c r="J34" s="1"/>
     </row>
     <row r="35" spans="2:13" x14ac:dyDescent="0.35">
@@ -4109,7 +4243,9 @@
       <c r="F35" s="16"/>
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
-      <c r="I35" s="1"/>
+      <c r="I35" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="J35" s="1"/>
     </row>
     <row r="36" spans="2:13" x14ac:dyDescent="0.35">
@@ -4122,10 +4258,10 @@
       <c r="F36" s="16"/>
       <c r="G36" s="16"/>
       <c r="H36" s="16"/>
-      <c r="I36" s="1"/>
-      <c r="J36" s="1">
-        <v>100000</v>
-      </c>
+      <c r="I36" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="1"/>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B37" s="16" t="s">
@@ -4137,7 +4273,9 @@
       <c r="F37" s="16"/>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
-      <c r="I37" s="1"/>
+      <c r="I37" s="1" t="n">
+        <v>5000</v>
+      </c>
       <c r="J37" s="1"/>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.35">
@@ -4153,11 +4291,11 @@
       <c r="I38" s="20"/>
       <c r="J38" s="8">
         <f>SUM(J24:J37)</f>
-        <v>171238.53611111111</v>
+        <v>217903.04187692306</v>
       </c>
       <c r="K38" s="9">
-        <f>J38/46000</f>
-        <v>3.7225768719806762</v>
+        <f>J38/B41</f>
+        <v>7.5138979957559675</v>
       </c>
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.35">
@@ -4173,8 +4311,8 @@
       <c r="I39" s="16"/>
       <c r="J39" s="16"/>
       <c r="K39" s="10">
-        <f>11500*(H13)/D20</f>
-        <v>6.2227777777777789</v>
+        <f>K12*H13/B41</f>
+        <v>10.351845711759504</v>
       </c>
       <c r="L39">
         <v>15800</v>
@@ -4202,45 +4340,47 @@
       </c>
       <c r="K40" s="12">
         <f>SUM(K38:K39)</f>
-        <v>9.9453546497584551</v>
+        <v>17.86574370751547</v>
       </c>
       <c r="L40" s="13">
         <f>K40*L39</f>
-        <v>157136.60346618359</v>
+        <v>282278.75057874445</v>
       </c>
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B41" s="16">
-        <v>45000</v>
+        <f>D20</f>
+        <v>29000</v>
       </c>
       <c r="C41" s="16"/>
       <c r="D41" s="16">
-        <v>20</v>
+        <f>ROUNDUP((J38+K12*H13)/B41,4)</f>
+        <v>17.8658</v>
       </c>
       <c r="E41" s="16"/>
       <c r="F41" s="16">
         <f>B41*D41</f>
-        <v>900000</v>
+        <v>518108.2</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16">
-        <f>F41*3.75%</f>
-        <v>33750</v>
+        <f>F41*0%</f>
+        <v>0</v>
       </c>
       <c r="I41" s="16"/>
       <c r="J41" s="1">
         <f>F41-H41</f>
-        <v>866250</v>
+        <v>518108.2</v>
       </c>
       <c r="K41" t="s">
         <v>73</v>
       </c>
-      <c r="L41" s="14">
-        <v>1.2500000000000001E-2</v>
+      <c r="L41" s="14" t="n">
+        <v>0</v>
       </c>
       <c r="M41" s="13">
         <f>F41*L41*L39</f>
-        <v>177750000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="2:13" x14ac:dyDescent="0.35">
@@ -4256,12 +4396,12 @@
       <c r="K42" t="s">
         <v>74</v>
       </c>
-      <c r="L42" s="14">
-        <v>2.5000000000000001E-2</v>
+      <c r="L42" s="14" t="n">
+        <v>0</v>
       </c>
       <c r="M42" s="13">
         <f>F41*L42*L39</f>
-        <v>355500000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="2:13" x14ac:dyDescent="0.35">
@@ -4290,29 +4430,29 @@
     <row r="44" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B44" s="19">
         <f>F41-J38</f>
-        <v>728761.46388888895</v>
+        <v>300205.15812307695</v>
       </c>
       <c r="C44" s="20"/>
       <c r="D44" s="21">
         <f>F41/H13</f>
-        <v>66529.774127310055</v>
+        <v>30202.488397294568</v>
       </c>
       <c r="E44" s="21"/>
-      <c r="F44" s="20">
-        <v>5612</v>
+      <c r="F44" s="20" t="n">
+        <v>6500</v>
       </c>
       <c r="G44" s="20"/>
       <c r="H44" s="4">
         <f>J41/H13</f>
-        <v>64034.90759753593</v>
+        <v>30202.488397294568</v>
       </c>
       <c r="I44" s="8">
         <f>J38/H13</f>
-        <v>12658.290143737166</v>
+        <v>12702.393233735658</v>
       </c>
       <c r="J44" s="8">
         <f>H44-F44-I44</f>
-        <v>45764.617453798768</v>
+        <v>11000.09516355891</v>
       </c>
     </row>
   </sheetData>

</xml_diff>